<commit_message>
Raise liquidity reserve and sync documents with the model
The model showed year 1 ending at 1.5 months of fixed costs with a
September trough of 21k EUR — below the plan's own 2.0 warning threshold.

- Liquidity reserve 60k -> 80k EUR, funded by raising the LfA tranche to
  252.3k. Year 1 now ends at 2.2 months, trough 40,254 EUR.
- Rewrote the financial plan document with the model's actual figures:
  investment 577.3k, capital need 657.3k, equity ratio 22.8%, EBITDA
  23/57/92/99/101k, cash flow -21/+14/+34/+22/+25k, break-even 46.2% with
  a 4.7 point margin over the year-3 plan.
- Added the debt service schedule and a note on why the reserve is 80k.
- Corrected the target KPI table in the business plan and the key figures
  in the README.

Model recalculated: 0 formula errors, funding gap 0 EUR.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DR8xtUwZtBi4pMv7HS3TGp
</commit_message>
<xml_diff>
--- a/padel-landshut/Finanzplan_Padel_Landshut.xlsx
+++ b/padel-landshut/Finanzplan_Padel_Landshut.xlsx
@@ -502,7 +502,7 @@
     <t xml:space="preserve">Liquiditätsreserve für die Anlaufphase</t>
   </si>
   <si>
-    <t xml:space="preserve">deckt den negativen Cashflow in Jahr 1</t>
+    <t xml:space="preserve">deckt Jahr 1 mit mind. 2 Monatsfixkosten Puffer</t>
   </si>
   <si>
     <t xml:space="preserve">Gesamtkapitalbedarf</t>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="I5" s="23" t="n">
         <f aca="false">G5-Finanzierung!$D$43</f>
-        <v>35147.5420168067</v>
+        <v>34247.5420168067</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="I6" s="23" t="n">
         <f aca="false">G6-Finanzierung!$D$43</f>
-        <v>-11055.2478991597</v>
+        <v>-11955.2478991597</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="I7" s="23" t="n">
         <f aca="false">G7-Finanzierung!$D$43</f>
-        <v>81350.3319327731</v>
+        <v>80450.3319327731</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="I8" s="23" t="n">
         <f aca="false">G8-Finanzierung!$D$43</f>
-        <v>20747.5420168067</v>
+        <v>19847.5420168067</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="I9" s="23" t="n">
         <f aca="false">G9-Finanzierung!$D$43</f>
-        <v>16877.5420168067</v>
+        <v>15977.5420168067</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="I10" s="23" t="n">
         <f aca="false">G10-Finanzierung!$D$43</f>
-        <v>7742.54201680679</v>
+        <v>6842.54201680679</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="I11" s="23" t="n">
         <f aca="false">G11-Finanzierung!$D$43</f>
-        <v>-43725.2478991597</v>
+        <v>-44625.2478991597</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3283,7 +3283,7 @@
         <v>156</v>
       </c>
       <c r="B21" s="22" t="n">
-        <v>60000</v>
+        <v>80000</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>157</v>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="B22" s="25" t="n">
         <f aca="false">B19+B21</f>
-        <v>637300</v>
+        <v>657300</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3433,7 +3433,7 @@
         <v>173</v>
       </c>
       <c r="B7" s="22" t="n">
-        <v>232300</v>
+        <v>252300</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>174</v>
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B9" s="23" t="n">
         <f aca="false">SUM(B4:B8)</f>
-        <v>637300</v>
+        <v>657300</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="B10" s="28" t="n">
         <f aca="false">Investition!B22</f>
-        <v>637300</v>
+        <v>657300</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="B12" s="29" t="n">
         <f aca="false">(B4+B5)/B9</f>
-        <v>0.235367958575239</v>
+        <v>0.228206298493838</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>180</v>
@@ -3542,7 +3542,7 @@
       </c>
       <c r="B17" s="27" t="n">
         <f aca="false">B7</f>
-        <v>232300</v>
+        <v>252300</v>
       </c>
       <c r="C17" s="15" t="n">
         <v>0.045</v>
@@ -3730,23 +3730,23 @@
       </c>
       <c r="B28" s="27" t="n">
         <f aca="false">B17</f>
-        <v>232300</v>
+        <v>252300</v>
       </c>
       <c r="C28" s="27" t="n">
         <f aca="false">B31</f>
-        <v>232300</v>
+        <v>252300</v>
       </c>
       <c r="D28" s="27" t="n">
         <f aca="false">C31</f>
-        <v>232300</v>
+        <v>252300</v>
       </c>
       <c r="E28" s="27" t="n">
         <f aca="false">D31</f>
-        <v>232300</v>
+        <v>252300</v>
       </c>
       <c r="F28" s="27" t="n">
         <f aca="false">E31</f>
-        <v>212941.666666667</v>
+        <v>231275</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3755,23 +3755,23 @@
       </c>
       <c r="B29" s="27" t="n">
         <f aca="false">B28*$C$17</f>
-        <v>10453.5</v>
+        <v>11353.5</v>
       </c>
       <c r="C29" s="27" t="n">
         <f aca="false">C28*$C$17</f>
-        <v>10453.5</v>
+        <v>11353.5</v>
       </c>
       <c r="D29" s="27" t="n">
         <f aca="false">D28*$C$17</f>
-        <v>10453.5</v>
+        <v>11353.5</v>
       </c>
       <c r="E29" s="27" t="n">
         <f aca="false">E28*$C$17</f>
-        <v>10453.5</v>
+        <v>11353.5</v>
       </c>
       <c r="F29" s="27" t="n">
         <f aca="false">F28*$C$17</f>
-        <v>9582.375</v>
+        <v>10407.375</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3792,11 +3792,11 @@
       </c>
       <c r="E30" s="27" t="n">
         <f aca="false">IF(4&lt;=$E$17,0,MIN(E28,$B$17/($D$17-$E$17)))</f>
-        <v>19358.3333333333</v>
+        <v>21025</v>
       </c>
       <c r="F30" s="27" t="n">
         <f aca="false">IF(5&lt;=$E$17,0,MIN(F28,$B$17/($D$17-$E$17)))</f>
-        <v>19358.3333333333</v>
+        <v>21025</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3805,23 +3805,23 @@
       </c>
       <c r="B31" s="27" t="n">
         <f aca="false">B28-B30</f>
-        <v>232300</v>
+        <v>252300</v>
       </c>
       <c r="C31" s="27" t="n">
         <f aca="false">C28-C30</f>
-        <v>232300</v>
+        <v>252300</v>
       </c>
       <c r="D31" s="27" t="n">
         <f aca="false">D28-D30</f>
-        <v>232300</v>
+        <v>252300</v>
       </c>
       <c r="E31" s="27" t="n">
         <f aca="false">E28-E30</f>
-        <v>212941.666666667</v>
+        <v>231275</v>
       </c>
       <c r="F31" s="27" t="n">
         <f aca="false">F28-F30</f>
-        <v>193583.333333333</v>
+        <v>210250</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3979,23 +3979,23 @@
       </c>
       <c r="B41" s="23" t="n">
         <f aca="false">B23+B29+B35</f>
-        <v>24503.5</v>
+        <v>25403.5</v>
       </c>
       <c r="C41" s="23" t="n">
         <f aca="false">C23+C29+C35</f>
-        <v>23389.2142857143</v>
+        <v>24289.2142857143</v>
       </c>
       <c r="D41" s="23" t="n">
         <f aca="false">D23+D29+D35</f>
-        <v>22274.9285714286</v>
+        <v>23174.9285714286</v>
       </c>
       <c r="E41" s="23" t="n">
         <f aca="false">E23+E29+E35</f>
-        <v>20379.3928571429</v>
+        <v>21279.3928571429</v>
       </c>
       <c r="F41" s="23" t="n">
         <f aca="false">F23+F29+F35</f>
-        <v>17612.7321428571</v>
+        <v>18437.7321428571</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4016,11 +4016,11 @@
       </c>
       <c r="E42" s="23" t="n">
         <f aca="false">E24+E30+E36</f>
-        <v>53554.7619047619</v>
+        <v>55221.4285714286</v>
       </c>
       <c r="F42" s="23" t="n">
         <f aca="false">F24+F30+F36</f>
-        <v>53554.7619047619</v>
+        <v>55221.4285714286</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4029,23 +4029,23 @@
       </c>
       <c r="B43" s="25" t="n">
         <f aca="false">B41+B42</f>
-        <v>43074.9285714286</v>
+        <v>43974.9285714286</v>
       </c>
       <c r="C43" s="25" t="n">
         <f aca="false">C41+C42</f>
-        <v>41960.6428571429</v>
+        <v>42860.6428571429</v>
       </c>
       <c r="D43" s="25" t="n">
         <f aca="false">D41+D42</f>
-        <v>56471.3571428571</v>
+        <v>57371.3571428571</v>
       </c>
       <c r="E43" s="25" t="n">
         <f aca="false">E41+E42</f>
-        <v>73934.1547619048</v>
+        <v>76500.8214285714</v>
       </c>
       <c r="F43" s="25" t="n">
         <f aca="false">F41+F42</f>
-        <v>71167.494047619</v>
+        <v>73659.1607142857</v>
       </c>
     </row>
   </sheetData>
@@ -5280,23 +5280,23 @@
       </c>
       <c r="B10" s="26" t="n">
         <f aca="false">-Finanzierung!B41</f>
-        <v>-24503.5</v>
+        <v>-25403.5</v>
       </c>
       <c r="C10" s="26" t="n">
         <f aca="false">-Finanzierung!C41</f>
-        <v>-23389.2142857143</v>
+        <v>-24289.2142857143</v>
       </c>
       <c r="D10" s="26" t="n">
         <f aca="false">-Finanzierung!D41</f>
-        <v>-22274.9285714286</v>
+        <v>-23174.9285714286</v>
       </c>
       <c r="E10" s="26" t="n">
         <f aca="false">-Finanzierung!E41</f>
-        <v>-20379.3928571429</v>
+        <v>-21279.3928571429</v>
       </c>
       <c r="F10" s="26" t="n">
         <f aca="false">-Finanzierung!F41</f>
-        <v>-17612.7321428571</v>
+        <v>-18437.7321428571</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5305,23 +5305,23 @@
       </c>
       <c r="B11" s="23" t="n">
         <f aca="false">B7+B9+B10</f>
-        <v>-51905.8268907563</v>
+        <v>-52805.8268907563</v>
       </c>
       <c r="C11" s="23" t="n">
         <f aca="false">C7+C9+C10</f>
-        <v>-16550.4487394958</v>
+        <v>-17450.4487394958</v>
       </c>
       <c r="D11" s="23" t="n">
         <f aca="false">D7+D9+D10</f>
-        <v>19118.8705882353</v>
+        <v>18218.8705882353</v>
       </c>
       <c r="E11" s="23" t="n">
         <f aca="false">E7+E9+E10</f>
-        <v>28168.8595378152</v>
+        <v>27268.8595378152</v>
       </c>
       <c r="F11" s="23" t="n">
         <f aca="false">F7+F9+F10</f>
-        <v>32935.3726388658</v>
+        <v>32110.3726388658</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5333,19 +5333,19 @@
       </c>
       <c r="C12" s="27" t="n">
         <f aca="false">B14</f>
-        <v>51905.8268907563</v>
+        <v>52805.8268907563</v>
       </c>
       <c r="D12" s="27" t="n">
         <f aca="false">C14</f>
-        <v>68456.275630252</v>
+        <v>70256.275630252</v>
       </c>
       <c r="E12" s="27" t="n">
         <f aca="false">D14</f>
-        <v>49337.4050420167</v>
+        <v>52037.4050420167</v>
       </c>
       <c r="F12" s="27" t="n">
         <f aca="false">E14</f>
-        <v>21168.5455042015</v>
+        <v>24768.5455042015</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5370,7 +5370,7 @@
       </c>
       <c r="F13" s="27" t="n">
         <f aca="false">-MAX(0,F11-F12)*Annahmen!$B$64</f>
-        <v>-3530.04814039928</v>
+        <v>-2202.54814039928</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5379,19 +5379,19 @@
       </c>
       <c r="B14" s="27" t="n">
         <f aca="false">MAX(0,B12-B11)</f>
-        <v>51905.8268907563</v>
+        <v>52805.8268907563</v>
       </c>
       <c r="C14" s="27" t="n">
         <f aca="false">MAX(0,C12-C11)</f>
-        <v>68456.275630252</v>
+        <v>70256.275630252</v>
       </c>
       <c r="D14" s="27" t="n">
         <f aca="false">MAX(0,D12-D11)</f>
-        <v>49337.4050420167</v>
+        <v>52037.4050420167</v>
       </c>
       <c r="E14" s="27" t="n">
         <f aca="false">MAX(0,E12-E11)</f>
-        <v>21168.5455042015</v>
+        <v>24768.5455042015</v>
       </c>
       <c r="F14" s="27" t="n">
         <f aca="false">MAX(0,F12-F11)</f>
@@ -5404,23 +5404,23 @@
       </c>
       <c r="B15" s="23" t="n">
         <f aca="false">B11+B13</f>
-        <v>-51905.8268907563</v>
+        <v>-52805.8268907563</v>
       </c>
       <c r="C15" s="23" t="n">
         <f aca="false">C11+C13</f>
-        <v>-16550.4487394958</v>
+        <v>-17450.4487394958</v>
       </c>
       <c r="D15" s="23" t="n">
         <f aca="false">D11+D13</f>
-        <v>19118.8705882353</v>
+        <v>18218.8705882353</v>
       </c>
       <c r="E15" s="23" t="n">
         <f aca="false">E11+E13</f>
-        <v>28168.8595378152</v>
+        <v>27268.8595378152</v>
       </c>
       <c r="F15" s="23" t="n">
         <f aca="false">F11+F13</f>
-        <v>29405.3244984665</v>
+        <v>29907.8244984665</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5482,23 +5482,23 @@
       </c>
       <c r="B20" s="26" t="n">
         <f aca="false">-Finanzierung!B43</f>
-        <v>-43074.9285714286</v>
+        <v>-43974.9285714286</v>
       </c>
       <c r="C20" s="26" t="n">
         <f aca="false">-Finanzierung!C43</f>
-        <v>-41960.6428571429</v>
+        <v>-42860.6428571429</v>
       </c>
       <c r="D20" s="26" t="n">
         <f aca="false">-Finanzierung!D43</f>
-        <v>-56471.3571428571</v>
+        <v>-57371.3571428571</v>
       </c>
       <c r="E20" s="26" t="n">
         <f aca="false">-Finanzierung!E43</f>
-        <v>-73934.1547619048</v>
+        <v>-76500.8214285714</v>
       </c>
       <c r="F20" s="26" t="n">
         <f aca="false">-Finanzierung!F43</f>
-        <v>-71167.494047619</v>
+        <v>-73659.1607142857</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5523,7 +5523,7 @@
       </c>
       <c r="F21" s="27" t="n">
         <f aca="false">F13</f>
-        <v>-3530.04814039928</v>
+        <v>-2202.54814039928</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5532,23 +5532,23 @@
       </c>
       <c r="B22" s="25" t="n">
         <f aca="false">B19+B20+B21</f>
-        <v>-20252.1554621849</v>
+        <v>-21152.1554621849</v>
       </c>
       <c r="C22" s="25" t="n">
         <f aca="false">C19+C20+C21</f>
-        <v>15103.2226890757</v>
+        <v>14203.2226890757</v>
       </c>
       <c r="D22" s="25" t="n">
         <f aca="false">D19+D20+D21</f>
-        <v>35147.5420168067</v>
+        <v>34247.5420168067</v>
       </c>
       <c r="E22" s="25" t="n">
         <f aca="false">E19+E20+E21</f>
-        <v>24839.1976330533</v>
+        <v>22272.5309663867</v>
       </c>
       <c r="F22" s="25" t="n">
         <f aca="false">F19+F20+F21</f>
-        <v>26075.6625937046</v>
+        <v>24911.4959270379</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5557,23 +5557,23 @@
       </c>
       <c r="B23" s="27" t="n">
         <f aca="false">B22</f>
-        <v>-20252.1554621849</v>
+        <v>-21152.1554621849</v>
       </c>
       <c r="C23" s="27" t="n">
         <f aca="false">B23+C22</f>
-        <v>-5148.93277310918</v>
+        <v>-6948.93277310918</v>
       </c>
       <c r="D23" s="27" t="n">
         <f aca="false">C23+D22</f>
-        <v>29998.6092436976</v>
+        <v>27298.6092436976</v>
       </c>
       <c r="E23" s="27" t="n">
         <f aca="false">D23+E22</f>
-        <v>54837.8068767509</v>
+        <v>49571.1402100842</v>
       </c>
       <c r="F23" s="27" t="n">
         <f aca="false">E23+F22</f>
-        <v>80913.4694704555</v>
+        <v>74482.6361371221</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5582,23 +5582,23 @@
       </c>
       <c r="B24" s="23" t="n">
         <f aca="false">Investition!$B$21+B22</f>
-        <v>39747.8445378151</v>
+        <v>58847.8445378151</v>
       </c>
       <c r="C24" s="23" t="n">
         <f aca="false">B24+C22</f>
-        <v>54851.0672268908</v>
+        <v>73051.0672268908</v>
       </c>
       <c r="D24" s="23" t="n">
         <f aca="false">C24+D22</f>
-        <v>89998.6092436976</v>
+        <v>107298.609243698</v>
       </c>
       <c r="E24" s="23" t="n">
         <f aca="false">D24+E22</f>
-        <v>114837.806876751</v>
+        <v>129571.140210084</v>
       </c>
       <c r="F24" s="23" t="n">
         <f aca="false">E24+F22</f>
-        <v>140913.469470455</v>
+        <v>154482.636137122</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>240</v>
@@ -5610,23 +5610,23 @@
       </c>
       <c r="B25" s="32" t="n">
         <f aca="false">IFERROR(B24/(Kosten!B17/12),0)</f>
-        <v>1.4982696229112</v>
+        <v>2.21823192854965</v>
       </c>
       <c r="C25" s="32" t="n">
         <f aca="false">IFERROR(C24/(Kosten!C17/12),0)</f>
-        <v>1.88816066185511</v>
+        <v>2.51466668595149</v>
       </c>
       <c r="D25" s="32" t="n">
         <f aca="false">IFERROR(D24/(Kosten!D17/12),0)</f>
-        <v>2.91565083711349</v>
+        <v>3.47611238097447</v>
       </c>
       <c r="E25" s="32" t="n">
         <f aca="false">IFERROR(E24/(Kosten!E17/12),0)</f>
-        <v>3.61461316095486</v>
+        <v>4.07835678354561</v>
       </c>
       <c r="F25" s="32" t="n">
         <f aca="false">IFERROR(F24/(Kosten!F17/12),0)</f>
-        <v>4.33458968760004</v>
+        <v>4.75198605235984</v>
       </c>
     </row>
   </sheetData>
@@ -5944,55 +5944,55 @@
       </c>
       <c r="B10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="C10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="D10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="E10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="F10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="G10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="H10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="I10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="J10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="K10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="L10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="M10" s="27" t="n">
         <f aca="false">-Finanzierung!$B$43/12</f>
-        <v>-3589.57738095238</v>
+        <v>-3664.57738095238</v>
       </c>
       <c r="N10" s="23" t="n">
         <f aca="false">SUM(B10:M10)</f>
-        <v>-43074.9285714286</v>
+        <v>-43974.9285714286</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6001,55 +6001,55 @@
       </c>
       <c r="B11" s="23" t="n">
         <f aca="false">SUM(B7:B10)</f>
-        <v>3998.53326330532</v>
+        <v>3923.53326330532</v>
       </c>
       <c r="C11" s="23" t="n">
         <f aca="false">SUM(C7:C10)</f>
-        <v>2292.66939775911</v>
+        <v>2217.66939775911</v>
       </c>
       <c r="D11" s="23" t="n">
         <f aca="false">SUM(D7:D10)</f>
-        <v>2292.66939775911</v>
+        <v>2217.66939775911</v>
       </c>
       <c r="E11" s="23" t="n">
         <f aca="false">SUM(E7:E10)</f>
-        <v>-2824.92219887955</v>
+        <v>-2899.92219887955</v>
       </c>
       <c r="F11" s="23" t="n">
         <f aca="false">SUM(F7:F10)</f>
-        <v>-6236.64992997199</v>
+        <v>-6311.64992997199</v>
       </c>
       <c r="G11" s="23" t="n">
         <f aca="false">SUM(G7:G10)</f>
-        <v>-9648.37766106443</v>
+        <v>-9723.37766106443</v>
       </c>
       <c r="H11" s="23" t="n">
         <f aca="false">SUM(H7:H10)</f>
-        <v>-13060.1053921569</v>
+        <v>-13135.1053921569</v>
       </c>
       <c r="I11" s="23" t="n">
         <f aca="false">SUM(I7:I10)</f>
-        <v>-13060.1053921569</v>
+        <v>-13135.1053921569</v>
       </c>
       <c r="J11" s="23" t="n">
         <f aca="false">SUM(J7:J10)</f>
-        <v>-2824.92219887955</v>
+        <v>-2899.92219887955</v>
       </c>
       <c r="K11" s="23" t="n">
         <f aca="false">SUM(K7:K10)</f>
-        <v>3998.53326330532</v>
+        <v>3923.53326330532</v>
       </c>
       <c r="L11" s="23" t="n">
         <f aca="false">SUM(L7:L10)</f>
-        <v>7410.26099439776</v>
+        <v>7335.26099439776</v>
       </c>
       <c r="M11" s="23" t="n">
         <f aca="false">SUM(M7:M10)</f>
-        <v>7410.26099439776</v>
+        <v>7335.26099439776</v>
       </c>
       <c r="N11" s="23" t="n">
         <f aca="false">SUM(B11:M11)</f>
-        <v>-20252.1554621849</v>
+        <v>-21152.1554621849</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6058,51 +6058,51 @@
       </c>
       <c r="B12" s="25" t="n">
         <f aca="false">Investition!$B$21+B11</f>
-        <v>63998.5332633053</v>
+        <v>83923.5332633053</v>
       </c>
       <c r="C12" s="25" t="n">
         <f aca="false">B12+C11</f>
-        <v>66291.2026610644</v>
+        <v>86141.2026610644</v>
       </c>
       <c r="D12" s="25" t="n">
         <f aca="false">C12+D11</f>
-        <v>68583.8720588235</v>
+        <v>88358.8720588235</v>
       </c>
       <c r="E12" s="25" t="n">
         <f aca="false">D12+E11</f>
-        <v>65758.949859944</v>
+        <v>85458.949859944</v>
       </c>
       <c r="F12" s="25" t="n">
         <f aca="false">E12+F11</f>
-        <v>59522.299929972</v>
+        <v>79147.299929972</v>
       </c>
       <c r="G12" s="25" t="n">
         <f aca="false">F12+G11</f>
-        <v>49873.9222689076</v>
+        <v>69423.9222689076</v>
       </c>
       <c r="H12" s="25" t="n">
         <f aca="false">G12+H11</f>
-        <v>36813.8168767507</v>
+        <v>56288.8168767507</v>
       </c>
       <c r="I12" s="25" t="n">
         <f aca="false">H12+I11</f>
-        <v>23753.7114845939</v>
+        <v>43153.7114845938</v>
       </c>
       <c r="J12" s="25" t="n">
         <f aca="false">I12+J11</f>
-        <v>20928.7892857143</v>
+        <v>40253.7892857143</v>
       </c>
       <c r="K12" s="25" t="n">
         <f aca="false">J12+K11</f>
-        <v>24927.3225490196</v>
+        <v>44177.3225490196</v>
       </c>
       <c r="L12" s="25" t="n">
         <f aca="false">K12+L11</f>
-        <v>32337.5835434174</v>
+        <v>51512.5835434174</v>
       </c>
       <c r="M12" s="25" t="n">
         <f aca="false">L12+M11</f>
-        <v>39747.8445378151</v>
+        <v>58847.8445378151</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="B14" s="23" t="n">
         <f aca="false">MIN(B12:M12)</f>
-        <v>20928.7892857143</v>
+        <v>40253.7892857143</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6181,7 +6181,7 @@
       </c>
       <c r="B5" s="26" t="n">
         <f aca="false">Finanzierung!D43</f>
-        <v>56471.3571428571</v>
+        <v>57371.3571428571</v>
       </c>
       <c r="D5" s="3"/>
     </row>
@@ -6191,7 +6191,7 @@
       </c>
       <c r="B6" s="23" t="n">
         <f aca="false">B4+B5</f>
-        <v>426880.357142857</v>
+        <v>427780.357142857</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6209,7 +6209,7 @@
       </c>
       <c r="B8" s="23" t="n">
         <f aca="false">B6+B7</f>
-        <v>336600.357142857</v>
+        <v>337500.357142857</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">IFERROR(B8/B9,0)</f>
-        <v>10639.0761195126</v>
+        <v>10667.5228169221</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="B12" s="31" t="n">
         <f aca="false">IFERROR(B10/B11,0)</f>
-        <v>0.460486327887493</v>
+        <v>0.461717573447113</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B14" s="33" t="n">
         <f aca="false">B13-B12</f>
-        <v>0.048083616710845</v>
+        <v>0.0468523711512248</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>279</v>

</xml_diff>